<commit_message>
Add external collaborator access and matter lifecycle status (US11)
Stakeholder requirements: external co-counsel access per matter + lifecycle status.

- Status model changed to Eval/Pre-Litigation/Litigation/Closed (one persistent Team+site; status is metadata) across the metadata model, content type, importer, and inventory templates.

- Grant-MatterExternalAccess.ps1: invite a guest and grant per-matter Team + SharePoint access (external access is inherently per-matter since each matter is its own group/site).

- Set-MatterStatus.ps1: change a matter's lifecycle status in place without recreating the Team; Closed flags for repository archival.

- New-MatterSite hardens sharing to ExternalUserSharingOnly (guests allowed, no anonymous links). Idempotent re-runs preserve status (no reset). Adds FR-023/024 and US11; runbook updated. Live guest+status validation (T070) pending a test guest.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/inventory/matter-inventory.template.xlsx
+++ b/inventory/matter-inventory.template.xlsx
@@ -62,7 +62,7 @@
     <t>MVA Personal Injury</t>
   </si>
   <si>
-    <t>Open</t>
+    <t>Litigation</t>
   </si>
   <si>
     <t>brennan@collinsattorneys.com</t>
@@ -157,7 +157,7 @@
     <col min="3" max="3" width="14.6739501953125" customWidth="1"/>
     <col min="4" max="4" width="18.74881935119629" customWidth="1"/>
     <col min="5" max="5" width="19.349079132080078" customWidth="1"/>
-    <col min="6" max="6" width="9.262957572937012" customWidth="1"/>
+    <col min="6" max="6" width="9.572667121887207" customWidth="1"/>
     <col min="7" max="7" width="28.966917037963867" customWidth="1"/>
     <col min="8" max="8" width="50.67942428588867" customWidth="1"/>
     <col min="9" max="9" width="24.66827392578125" customWidth="1"/>
@@ -237,8 +237,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="F2:F1000" showErrorMessage="1" errorTitle="Invalid Status" error="Status must be Prospective, Open, Closed, or Intake.">
-      <formula1>"Prospective,Open,Closed,Intake"</formula1>
+    <dataValidation type="list" sqref="F2:F1000" showErrorMessage="1" errorTitle="Invalid Status" error="Status must be Eval, Pre-Litigation, Litigation, or Closed.">
+      <formula1>"Eval,Pre-Litigation,Litigation,Closed"</formula1>
     </dataValidation>
   </dataValidations>
   <headerFooter/>

</xml_diff>